<commit_message>
updated building template; update index landing page updated figure of basic overview;
</commit_message>
<xml_diff>
--- a/overview/PMO_building_template.xlsx
+++ b/overview/PMO_building_template.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nicholashathaway/projects/plasmodium/falciparum/Portable_Microhaplotype_Object_Tools/overview/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nicholashathaway/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AF6249E-BF40-4B46-946A-D99A07D987CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F7D3550-979F-9142-B885-1E5B71D5FBB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="17" r:id="rId1"/>
     <sheet name="Required Panel Targets " sheetId="3" r:id="rId2"/>
     <sheet name="Required Panel Info" sheetId="15" r:id="rId3"/>
-    <sheet name="Optional GenomeInfo" sheetId="6" r:id="rId4"/>
-    <sheet name="Required Microhaplotype" sheetId="1" r:id="rId5"/>
+    <sheet name="Required Microhaplotype" sheetId="1" r:id="rId4"/>
+    <sheet name="Optional GenomeInfo" sheetId="6" r:id="rId5"/>
     <sheet name="Optional Specimen Level" sheetId="7" r:id="rId6"/>
     <sheet name="Optional ProjectInfo" sheetId="11" r:id="rId7"/>
     <sheet name="Optional LibrarySampleInfo" sheetId="13" r:id="rId8"/>
@@ -34,6 +34,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
+    <author>Microsoft Office User</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000007000000}">
@@ -75,7 +76,33 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000002000000}">
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000002000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>a list of 1 or more reactions that this panel contains, each reactions list the targets that were amplified in that reaction, e.g. pool1, pool2</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000001000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>a name for the panel</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000002000000}">
       <text>
         <r>
           <rPr>
@@ -88,7 +115,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000003000000}">
+    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000003000000}">
       <text>
         <r>
           <rPr>
@@ -101,7 +128,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000004000000}">
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000004000000}">
       <text>
         <r>
           <rPr>
@@ -114,7 +141,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000006000000}">
+    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000006000000}">
       <text>
         <r>
           <rPr>
@@ -127,29 +154,16 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>a list of 1 or more reactions that this panel contains, each reactions list the targets that were amplified in that reaction, e.g. pool1, pool2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>a name for the panel</t>
+    <comment ref="J1" authorId="1" shapeId="0" xr:uid="{C0C2BF61-21CA-2649-B7CD-8A70648DE04F}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>fields not yet defined by the PMO schema that a user wants to include with their data</t>
         </r>
       </text>
     </comment>
@@ -161,6 +175,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
+    <author>Microsoft Office User</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0" xr:uid="{6410ADFB-0FE7-1D4A-B78B-1C40BD1C9E2A}">
@@ -186,6 +201,19 @@
             <family val="2"/>
           </rPr>
           <t>the date when the run was done, should be YYYY-MM-DD</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="1" shapeId="0" xr:uid="{A32DE3DB-79FF-8B43-8C46-555FB57CCED2}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>fields not yet defined by the PMO schema that a user wants to include with their data</t>
         </r>
       </text>
     </comment>
@@ -197,6 +225,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
+    <author>Microsoft Office User</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000004000000}">
@@ -287,6 +316,19 @@
             <family val="2"/>
           </rPr>
           <t>which strand the location is, either + for plus strand or - for negative strand</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="1" shapeId="0" xr:uid="{38A994C9-9C34-9641-8525-B0B01315D6CF}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>fields not yet defined by the PMO schema that a user wants to include with their data</t>
         </r>
       </text>
     </comment>
@@ -298,6 +340,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
+    <author>Microsoft Office User</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0" xr:uid="{14B36319-E81A-954D-A83E-2C73318DC5F8}">
@@ -336,6 +379,19 @@
             <family val="2"/>
           </rPr>
           <t>a name for this reaction</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="1" shapeId="0" xr:uid="{A7530953-2C5B-C443-A090-09A0088E3ABE}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>fields not yet defined by the PMO schema that a user wants to include with their data</t>
         </r>
       </text>
     </comment>
@@ -347,83 +403,188 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
+    <author>Microsoft Office User</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000004000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>name of the genome</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>the genome version</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000005000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>the NCBI taxonomy number, can be a list of values if it's a genome file that has been created by combining gnomes from different species</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000006000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>a link to the where this genome file could be downloaded</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>a list of the chromosomes/contigs found within this genome</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>a link to the where this genome's annotation file could be downloaded</t>
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{271ABD85-EC66-6241-AAAD-441A26D861B3}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>a unique identifier for this sequencing/amplification run</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{ABC44844-5D2A-1049-90EF-2078D540CAE8}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>a name for this target</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>the sequence</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>the read count for this microhaplotype</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{8BC4F583-6FE7-2645-A888-2434AA7C0D17}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">a name to for this run, needs to be unique to each run </t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000003000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>the unique molecular identifier (umi) count for this microhaplotype</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>a list of additional annotations associated with this microhaplotype, e.g. wildtype</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>a list of protein variants for this haplotype, e.g. amino acid changes/INDELS</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>a list of sequence variants for this haplotype, e.g. SNPS, indels</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>masking info for the sequence</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>an optional name for this microhaplotype</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>the pseudocigar of the haplotype</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>the ASCII fastq per base quality score for this sequence, this is optional, must be same length as the sequence</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="1" shapeId="0" xr:uid="{35EE2F69-AB1B-D44A-B152-6B9F532C3390}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>fields not yet defined by the PMO schema that a user wants to include with their data</t>
         </r>
       </text>
     </comment>
@@ -435,174 +596,97 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
+    <author>Microsoft Office User</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{271ABD85-EC66-6241-AAAD-441A26D861B3}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>a unique identifier for this sequencing/amplification run</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{ABC44844-5D2A-1049-90EF-2078D540CAE8}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>a name for this target</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>the sequence</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>the read count for this microhaplotype</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{8BC4F583-6FE7-2645-A888-2434AA7C0D17}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">a name to for this run, needs to be unique to each run </t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>the unique molecular identifier (umi) count for this microhaplotype</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>a list of additional annotations associated with this microhaplotype, e.g. wildtype</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>a list of protein variants for this haplotype, e.g. amino acid changes/INDELS</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>a list of sequence variants for this haplotype, e.g. SNPS, indels</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>masking info for the sequence</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>an optional name for this microhaplotype</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>the pseudocigar of the haplotype</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-          </rPr>
-          <t>the ASCII fastq per base quality score for this sequence, this is optional, must be same length as the sequence</t>
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000004000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>name of the genome</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000002000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>the genome version</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000005000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>the NCBI taxonomy number, can be a list of values if it's a genome file that has been created by combining gnomes from different species</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000006000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>a link to the where this genome file could be downloaded</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000001000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>a list of the chromosomes/contigs found within this genome</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000003000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>a link to the where this genome's annotation file could be downloaded</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="1" shapeId="0" xr:uid="{C07F9AB3-6586-D048-8BD9-F50560C60AD3}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>fields not yet defined by the PMO schema that a user wants to include with their data</t>
         </r>
       </text>
     </comment>
@@ -614,6 +698,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
+    <author>Microsoft Office User</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0600-000018000000}">
@@ -1016,6 +1101,19 @@
             <family val="2"/>
           </rPr>
           <t>If person has been treated with drugs, what was the treatment outcome</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AF1" authorId="1" shapeId="0" xr:uid="{30A07F9E-181B-AD47-A49D-B15C4FC6DD9E}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>fields not yet defined by the PMO schema that a user wants to include with their data</t>
         </r>
       </text>
     </comment>
@@ -1027,6 +1125,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
+    <author>Microsoft Office User</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0A00-000005000000}">
@@ -1104,6 +1203,19 @@
             <family val="2"/>
           </rPr>
           <t>the type of project conducted, e.g. TES vs surveillance vs transmission</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="1" shapeId="0" xr:uid="{7C8CE86E-7BFA-CC40-BE46-C749246F73A9}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>fields not yet defined by the PMO schema that a user wants to include with their data</t>
         </r>
       </text>
     </comment>
@@ -1115,6 +1227,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
+    <author>Microsoft Office User</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0C00-000005000000}">
@@ -1244,6 +1357,19 @@
             <family val="2"/>
           </rPr>
           <t>ERA/SRA run accession number for the sample if it was submitted</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="1" shapeId="0" xr:uid="{2C03E27F-E7D4-F849-B618-472D7C860CCE}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>fields not yet defined by the PMO schema that a user wants to include with their data</t>
         </r>
       </text>
     </comment>
@@ -1255,6 +1381,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
+    <author>Microsoft Office User</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0B00-000010000000}">
@@ -1462,6 +1589,19 @@
             <family val="2"/>
           </rPr>
           <t>the date of sequencing, should be YYYY-MM or YYYY-MM-DD</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="1" shapeId="0" xr:uid="{E7B54FCC-88B5-4545-826C-E81C3F99724B}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>fields not yet defined by the PMO schema that a user wants to include with their data</t>
         </r>
       </text>
     </comment>
@@ -1473,6 +1613,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
+    <author>Microsoft Office User</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0" xr:uid="{84E6B4A2-A3D7-2545-B916-A9C6570858E3}">
@@ -1537,6 +1678,19 @@
             <family val="2"/>
           </rPr>
           <t>a url pointing to code base of a program, e.g. a github link</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="1" shapeId="0" xr:uid="{6477AD37-0492-1443-85F4-C51EB8CC7D2F}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>fields not yet defined by the PMO schema that a user wants to include with their data</t>
         </r>
       </text>
     </comment>
@@ -1545,7 +1699,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="142">
   <si>
     <t>seq</t>
   </si>
@@ -1844,12 +1998,6 @@
     <t>Overview</t>
   </si>
   <si>
-    <t xml:space="preserve">This page describes what is in this template for building a Portable Microhaplotype Object (PMO)  </t>
-  </si>
-  <si>
-    <t>Found more details at: https://plasmogenepi.github.io/PMO_Docs/</t>
-  </si>
-  <si>
     <t>Page</t>
   </si>
   <si>
@@ -1865,9 +2013,6 @@
     <t>Not Required In Format</t>
   </si>
   <si>
-    <t>Not defined by schema, (custom fields are allowed)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Required Panel Targets </t>
   </si>
   <si>
@@ -1901,38 +2046,180 @@
     <t>In the target info has genomic location info, have to have meta data on the targeted genomes</t>
   </si>
   <si>
-    <t>Required information on the panel, panel_name at minimum</t>
-  </si>
-  <si>
-    <t>Required information on the panel's target, at minimum: target_name, forward_primer, reverse_primer</t>
-  </si>
-  <si>
-    <t>Required Information on the detected microhaplotypes, at minimum: library_sample_name, target_name, seq, reads</t>
-  </si>
-  <si>
-    <t>Optional meta data on the samples (in PMO called specimens)</t>
-  </si>
-  <si>
-    <t>Optional meta data on the project that samples belong to</t>
-  </si>
-  <si>
-    <t>Optional meta data on the seqeuncing of samples (each specimen might have multiple sequencing run, each run is refrered as a library_sample)</t>
-  </si>
-  <si>
-    <t>Optional meta on the seqeuncing info, this includes date, what type of machine (e.g. Illumina etc)</t>
-  </si>
-  <si>
-    <t>Optional meta data on the methods used to generate the detected microahaplotypes</t>
-  </si>
-  <si>
-    <t>Optional meta data on the various different bioinformatics runs if samples were analayzed all in one call or in multiple</t>
+    <t>Information on the panel</t>
+  </si>
+  <si>
+    <t>Information on the panel's target</t>
+  </si>
+  <si>
+    <t>Required Information on the detected microhaplotypes</t>
+  </si>
+  <si>
+    <t>Meta data on the samples (in PMO called specimens)</t>
+  </si>
+  <si>
+    <t>Meta data on the project that samples belong to</t>
+  </si>
+  <si>
+    <t>Meta data on the seqeuncing of samples (each specimen might have multiple sequencing run, each run is refrered as a library_sample)</t>
+  </si>
+  <si>
+    <t>Meta on the seqeuncing info, this includes date, what type of machine (e.g. Illumina etc)</t>
+  </si>
+  <si>
+    <t>Meta data on the methods used to generate the detected microahaplotypes</t>
+  </si>
+  <si>
+    <t>Meta data on the various different bioinformatics runs if samples were analayzed all in one call or in multiple</t>
+  </si>
+  <si>
+    <t>panel_info</t>
+  </si>
+  <si>
+    <t>target_info,panel_info</t>
+  </si>
+  <si>
+    <t>representative_microhaplotypes,detected_microhaplotypes</t>
+  </si>
+  <si>
+    <t>targeted_genomes</t>
+  </si>
+  <si>
+    <t>specimen_info</t>
+  </si>
+  <si>
+    <t>project_info</t>
+  </si>
+  <si>
+    <t>library_sample_info</t>
+  </si>
+  <si>
+    <t>sequencing_info</t>
+  </si>
+  <si>
+    <t>bioinformatics_methods_info</t>
+  </si>
+  <si>
+    <t>bioinformatics_run_info</t>
+  </si>
+  <si>
+    <t>This template provides a structured format for building a Portable Microhaplotype Object (PMO).</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The template contains separate </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>required</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>optional</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> sheets, along with the fields defined by the PMO specification. Required fields must be completed to create a valid PMO, while optional fields can be used to store additional metadata. Hover over red triangle in field cells to view descriptions and guidance for each field.</t>
+    </r>
+  </si>
+  <si>
+    <t>In addition to the standard PMO fields, you may add your own custom fields to store project-specific information. If there are fields that you use regularly and believe would be broadly useful to the community, please contact us and we can consider incorporating them into a future version of the PMO specification.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The template can be used as a reference for understanding the PMO structure or completed directly and imported into </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PMO App</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> or </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>pmotools-python</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to generate a PMO file. (CAUTION: Ensure dates are stored as YYYY-MM-DD format)</t>
+    </r>
+  </si>
+  <si>
+    <t>Not defined by schema, (custom fields are allowed, but not recommended)</t>
+  </si>
+  <si>
+    <t>custom_field</t>
+  </si>
+  <si>
+    <t>Associated PMO Sections</t>
+  </si>
+  <si>
+    <t>Find more details at: https://plasmogenepi.github.io/PMO_Docs/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1941,29 +2228,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF276221"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF833C00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="9"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF833B00"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1984,9 +2250,32 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color rgb="FF266221"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1994,7 +2283,14 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF833B00"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2009,34 +2305,36 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFCE4D7"/>
+        <fgColor rgb="FFDDEE3B"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
+        <fgColor rgb="FFFCDAE7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor rgb="FF7589C3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCDAE6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7589C4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -2045,35 +2343,144 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2083,10 +2490,16 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFCDAE6"/>
+      <color rgb="FFDDEE3B"/>
+      <color rgb="FF7589C4"/>
+      <color rgb="FF53B150"/>
+      <color rgb="FF000000"/>
+      <color rgb="FF7589C3"/>
+      <color rgb="FFFCDAE7"/>
+      <color rgb="FF92CEDC"/>
       <color rgb="FF833B00"/>
       <color rgb="FFFCE4D7"/>
-      <color rgb="FF266221"/>
-      <color rgb="FFC6EFCE"/>
     </mruColors>
   </colors>
   <extLst>
@@ -2379,133 +2792,183 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0E6E16-98CE-9440-B72E-D14072BA8199}">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="75.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="100.5" customWidth="1"/>
+    <col min="3" max="3" width="47.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="64" x14ac:dyDescent="0.2">
+      <c r="A5" s="23" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="48" x14ac:dyDescent="0.2">
+      <c r="A6" s="23" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="64" x14ac:dyDescent="0.2">
+      <c r="A7" s="23" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="18" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="19" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="7" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="8" t="s">
         <v>99</v>
       </c>
+      <c r="B17" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>140</v>
+      </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="5" t="s">
-        <v>100</v>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>125</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
-        <v>103</v>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="B19" t="s">
+        <v>115</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>124</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
-        <v>104</v>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="B20" t="s">
+        <v>117</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>126</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="8" t="s">
-        <v>105</v>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="B21" t="s">
+        <v>114</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>127</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="6" t="s">
-        <v>106</v>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="B22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>128</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>102</v>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="B23" t="s">
+        <v>119</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>129</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="B11" t="s">
-        <v>119</v>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="B24" t="s">
+        <v>120</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>130</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="B12" t="s">
-        <v>118</v>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B25" t="s">
+        <v>121</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>131</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="B13" t="s">
-        <v>117</v>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="B26" t="s">
+        <v>122</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>132</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="B14" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="B15" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="B16" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="8" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B27" s="16" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="B18" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="B19" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="B20" t="s">
-        <v>126</v>
+      <c r="C27" s="17" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -2518,7 +2981,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.1640625" bestFit="1" customWidth="1"/>
@@ -2529,21 +2992,24 @@
     <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="21" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="21" t="s">
         <v>94</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2555,19 +3021,22 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34F96FFD-ED84-7249-8E2D-AF60EFEAC77B}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.1640625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="22" t="s">
         <v>96</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2578,7 +3047,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.83203125" bestFit="1" customWidth="1"/>
@@ -2590,27 +3059,30 @@
     <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="21" t="s">
         <v>25</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2622,47 +3094,50 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>18</v>
+      <c r="J1" s="6" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2674,23 +3149,26 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A98C645F-2B46-3346-9A27-A1B971053D40}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1640625" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="20" t="s">
         <v>97</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2700,48 +3178,8 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="4.6640625" customWidth="1"/>
-    <col min="2" max="2" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="8.6640625" customWidth="1"/>
-    <col min="4" max="4" width="3.6640625" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" customWidth="1"/>
-    <col min="6" max="6" width="7.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <legacyDrawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.83203125" bestFit="1" customWidth="1"/>
@@ -2759,45 +3197,91 @@
     <col min="13" max="13" width="6.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A1" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="21" t="s">
         <v>7</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="4.6640625" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="8.6640625" customWidth="1"/>
+    <col min="4" max="4" width="3.6640625" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+    <col min="6" max="6" width="7.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2809,7 +3293,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AF1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.83203125" bestFit="1" customWidth="1"/>
@@ -2817,7 +3301,7 @@
     <col min="3" max="3" width="17.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.33203125" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.83203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.1640625" bestFit="1" customWidth="1"/>
@@ -2842,101 +3326,105 @@
     <col min="29" max="29" width="15.5" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="18.1640625" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="8.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A1" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="V1" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="W1" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="X1" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Y1" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="Z1" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AA1" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AB1" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AC1" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AD1" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AE1" s="21" t="s">
         <v>61</v>
+      </c>
+      <c r="AF1" s="6" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2948,7 +3436,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.6640625" customWidth="1"/>
@@ -2959,24 +3447,27 @@
     <col min="6" max="6" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="21" t="s">
         <v>67</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2988,7 +3479,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.83203125" bestFit="1" customWidth="1"/>
@@ -3003,36 +3494,39 @@
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="21" t="s">
         <v>85</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="21" t="s">
         <v>89</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -3044,7 +3538,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.6640625" customWidth="1"/>
@@ -3062,57 +3556,60 @@
     <col min="13" max="13" width="18.6640625" customWidth="1"/>
     <col min="14" max="14" width="8.6640625" customWidth="1"/>
     <col min="15" max="15" width="10.6640625" customWidth="1"/>
-    <col min="16" max="16" width="8.6640625" customWidth="1"/>
+    <col min="16" max="16" width="8.6640625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A1" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="22" t="s">
         <v>83</v>
+      </c>
+      <c r="Q1" s="6" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>